<commit_message>
Update people, navbar, news
</commit_message>
<xml_diff>
--- a/event_list.xlsx
+++ b/event_list.xlsx
@@ -122,7 +122,7 @@
     <xf fontId="1" fillId="0" borderId="0" numFmtId="9" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyProtection="0">
       <protection hidden="0" locked="1"/>
     </xf>
@@ -135,19 +135,11 @@
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top"/>
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="14" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top"/>
-      <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1" applyProtection="0">
-      <alignment vertical="top" wrapText="1"/>
       <protection hidden="0" locked="1"/>
     </xf>
   </cellXfs>
@@ -662,9 +654,9 @@
     </row>
     <row r="2" ht="12.75">
       <c r="A2" s="2">
-        <v>46353</v>
-      </c>
-      <c r="B2" s="3" t="s">
+        <v>46699</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -676,12 +668,12 @@
       <c r="E2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="3" t="s">
         <v>13</v>
       </c>
       <c r="G2" s="1">
         <f>DAY(A2)</f>
-        <v>27</v>
+        <v>8</v>
       </c>
       <c r="H2" s="2" t="str">
         <f>UPPER(TEXT(A2,"mmm"))</f>
@@ -689,16 +681,16 @@
       </c>
       <c r="I2" s="1">
         <f>YEAR(A2)</f>
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="J2"/>
     </row>
-    <row r="3" ht="102">
-      <c r="A3" s="5">
-        <v>46326</v>
+    <row r="3" ht="12.75">
+      <c r="A3" s="2">
+        <v>46560</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>10</v>
@@ -709,28 +701,29 @@
       <c r="E3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="3" t="s">
         <v>13</v>
       </c>
       <c r="G3" s="1">
-        <f t="shared" ref="G3:G9" si="0">DAY(A3)</f>
-        <v>31</v>
-      </c>
-      <c r="H3" s="5" t="str">
-        <f t="shared" ref="H3:H9" si="1">UPPER(TEXT(A3,"mmm"))</f>
-        <v>OCT</v>
+        <f>DAY(A3)</f>
+        <v>22</v>
+      </c>
+      <c r="H3" s="2" t="str">
+        <f>UPPER(TEXT(A3,"mmm"))</f>
+        <v>JUN</v>
       </c>
       <c r="I3" s="1">
-        <f t="shared" ref="I3:I9" si="2">YEAR(A3)</f>
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="4" ht="102">
-      <c r="A4" s="5">
-        <v>46322</v>
+        <f>YEAR(A3)</f>
+        <v>2027</v>
+      </c>
+      <c r="J3"/>
+    </row>
+    <row r="4" ht="12.75">
+      <c r="A4" s="2">
+        <v>46527</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>10</v>
@@ -741,156 +734,158 @@
       <c r="E4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="3" t="s">
         <v>13</v>
       </c>
       <c r="G4" s="1">
+        <f>DAY(A4)</f>
+        <v>20</v>
+      </c>
+      <c r="H4" s="2" t="str">
+        <f>UPPER(TEXT(A4,"mmm"))</f>
+        <v>MAY</v>
+      </c>
+      <c r="I4" s="1">
+        <f>YEAR(A4)</f>
+        <v>2027</v>
+      </c>
+      <c r="J4"/>
+    </row>
+    <row r="5" ht="102">
+      <c r="A5" s="4">
+        <v>46353</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G5" s="1">
+        <f>DAY(A5)</f>
+        <v>27</v>
+      </c>
+      <c r="H5" s="4" t="str">
+        <f>UPPER(TEXT(A5,"mmm"))</f>
+        <v>NOV</v>
+      </c>
+      <c r="I5" s="1">
+        <f>YEAR(A5)</f>
+        <v>2026</v>
+      </c>
+      <c r="J5"/>
+    </row>
+    <row r="6" ht="102">
+      <c r="A6" s="4">
+        <v>46326</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G6" s="1">
+        <f t="shared" ref="G6:G12" si="0">DAY(A6)</f>
+        <v>31</v>
+      </c>
+      <c r="H6" s="4" t="str">
+        <f t="shared" ref="H6:H12" si="1">UPPER(TEXT(A6,"mmm"))</f>
+        <v>OCT</v>
+      </c>
+      <c r="I6" s="1">
+        <f t="shared" ref="I6:I12" si="2">YEAR(A6)</f>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="7" ht="102">
+      <c r="A7" s="4">
+        <v>46322</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G7" s="1">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="H4" s="5" t="str">
+      <c r="H7" s="4" t="str">
         <f t="shared" si="1"/>
         <v>OCT</v>
       </c>
-      <c r="I4" s="1">
+      <c r="I7" s="1">
         <f t="shared" si="2"/>
         <v>2026</v>
       </c>
     </row>
-    <row r="5" ht="102">
-      <c r="A5" s="5">
+    <row r="8" ht="102">
+      <c r="A8" s="4">
         <v>46283</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G5" s="1">
+      <c r="G8" s="1">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="H5" s="5" t="str">
+      <c r="H8" s="4" t="str">
         <f t="shared" si="1"/>
         <v>SEP</v>
-      </c>
-      <c r="I5" s="1">
-        <f t="shared" si="2"/>
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="6" ht="90" customHeight="1">
-      <c r="A6" s="5">
-        <v>46285</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" s="1">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="H6" s="5" t="str">
-        <f t="shared" si="1"/>
-        <v>SEP</v>
-      </c>
-      <c r="I6" s="1">
-        <f t="shared" si="2"/>
-        <v>2026</v>
-      </c>
-    </row>
-    <row r="7" ht="102">
-      <c r="A7" s="5">
-        <v>45981</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G7" s="1">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="H7" s="5" t="str">
-        <f t="shared" si="1"/>
-        <v>NOV</v>
-      </c>
-      <c r="I7" s="1">
-        <f t="shared" si="2"/>
-        <v>2025</v>
-      </c>
-    </row>
-    <row r="8" ht="102">
-      <c r="A8" s="5">
-        <v>46078</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G8" s="1">
-        <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-      <c r="H8" s="5" t="str">
-        <f t="shared" si="1"/>
-        <v>FEB</v>
       </c>
       <c r="I8" s="1">
         <f t="shared" si="2"/>
         <v>2026</v>
       </c>
     </row>
-    <row r="9" ht="102">
-      <c r="A9" s="5">
-        <v>46174</v>
+    <row r="9" ht="90" customHeight="1">
+      <c r="A9" s="4">
+        <v>46285</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>10</v>
@@ -901,18 +896,114 @@
       <c r="E9" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="6" t="s">
+      <c r="F9" s="3" t="s">
         <v>13</v>
       </c>
       <c r="G9" s="1">
         <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="H9" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>SEP</v>
+      </c>
+      <c r="I9" s="1">
+        <f t="shared" si="2"/>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="10" ht="102">
+      <c r="A10" s="4">
+        <v>45981</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="1">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="H10" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>NOV</v>
+      </c>
+      <c r="I10" s="1">
+        <f t="shared" si="2"/>
+        <v>2025</v>
+      </c>
+    </row>
+    <row r="11" ht="102">
+      <c r="A11" s="4">
+        <v>46078</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G11" s="1">
+        <f t="shared" si="0"/>
+        <v>25</v>
+      </c>
+      <c r="H11" s="4" t="str">
+        <f t="shared" si="1"/>
+        <v>FEB</v>
+      </c>
+      <c r="I11" s="1">
+        <f t="shared" si="2"/>
+        <v>2026</v>
+      </c>
+    </row>
+    <row r="12" ht="102">
+      <c r="A12" s="4">
+        <v>46174</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="G12" s="1">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="H9" s="5" t="str">
+      <c r="H12" s="4" t="str">
         <f t="shared" si="1"/>
         <v>JUN</v>
       </c>
-      <c r="I9" s="1">
+      <c r="I12" s="1">
         <f t="shared" si="2"/>
         <v>2026</v>
       </c>

</xml_diff>